<commit_message>
Publish Duisburg_2018_WC, Montemor_2018_WCH, Plovdiv_2018_JWCH, Szeged_2018_WC, VilaVerde_2018_MAR
</commit_message>
<xml_diff>
--- a/events/VilaVerde_2018_MAR/VilaVerde_2018_MAR_Results.xlsx
+++ b/events/VilaVerde_2018_MAR/VilaVerde_2018_MAR_Results.xlsx
@@ -15377,6 +15377,11 @@
           <t>02:07:08.730</t>
         </is>
       </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -22306,7 +22311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D317"/>
+  <dimension ref="A1:D318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29283,6 +29288,28 @@
         </is>
       </c>
     </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>BEDEC</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>